<commit_message>
Corte SD: una S02 mas, entregada dentro de la ventana de tarde
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S04-corte-12sep.xlsx
+++ b/calificaciones/P00-S04-corte-12sep.xlsx
@@ -746,31 +746,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -778,7 +778,7 @@
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>Ya hiciste tu primer push. Falta toda la S02.</t>
+          <t>Completa. Llego tarde pero dentro de la ventana, y esta bien hecha: no te falta nada de la S02.</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
     <row r="54">
       <c r="A54" s="15" t="inlineStr">
         <is>
-          <t>S02 completa: 37 / 43   ·   parcial: 2   ·   sin entregar: 4</t>
+          <t>S02 completa: 38 / 43   ·   parcial: 2   ·   sin entregar: 3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corte SD 12-sep: la S02 de 321132477 si estaba entregada, se retira su hoja y una observacion deja de nombrar una carpeta
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S04-corte-12sep.xlsx
+++ b/calificaciones/P00-S04-corte-12sep.xlsx
@@ -8,15 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="Matriz" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="321132477" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="320298835" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="320152841" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="320250648" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="319659852" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="320229264" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="320284858" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="320224159" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="320049376" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="320298835" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="320152841" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="320250648" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="319659852" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="320229264" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="320284858" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="320224159" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="320049376" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -641,6 +640,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -840,31 +840,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>tarde</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>tarde</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -872,7 +872,7 @@
       </c>
       <c r="I10" s="10" t="inlineStr">
         <is>
-          <t>Tus lecturas SI estan registradas. Falta la S02: cuando la subas se actualiza.</t>
+          <t>Completa. Tu S02 si llego, se nos habia pasado: esta bien hecha y es de las mas completas. Detalle menor: tu p00 quedo en latin-1 y tu apellido sale con caracteres raros.</t>
         </is>
       </c>
     </row>
@@ -2756,6 +2756,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="14" t="inlineStr">
         <is>
@@ -2773,7 +2774,7 @@
     <row r="54">
       <c r="A54" s="15" t="inlineStr">
         <is>
-          <t>S02 completa: 38 / 43   ·   parcial: 2   ·   sin entregar: 3</t>
+          <t>S02 completa: 39 / 43   ·   parcial: 2   ·   sin entregar: 2</t>
         </is>
       </c>
     </row>
@@ -2809,125 +2810,6 @@
       <c r="A59" s="15" t="inlineStr">
         <is>
           <t>Idempotency key (tarea extra): 0 / 43 — sigue abierta, es opcional y no afecta la calificacion</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
-          <t>Correccion · 320049376</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320049376   ·   Por corregir: p00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>P00: ✓      S02: ✓      L2: ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>No tienes p00, que era la primera tarea de Git.</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Crea entregas/tu_carpeta/p00/prueba.txt con tu nombre completo adentro y haz push. Tu S02 si esta completa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="20" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="20" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="20" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="20" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="20" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
       </c>
     </row>
@@ -2952,24 +2834,25 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 321132477</t>
+          <t>Correccion · 320298835</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 321132477   ·   Por corregir: S02</t>
+          <t>Cuenta: 320298835   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: ✗      L2: tarde</t>
-        </is>
-      </c>
-    </row>
+          <t>P00: ✓      S02: ✓      L2: ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
@@ -2985,27 +2868,28 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>No subiste nada de la S02: falta el Dockerfile, el index.html y la evidencia.md.</t>
+          <t>Tu p00 no lleva tu nombre: dice 'esta es una prueba de git'.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>La guia del lab esta en labs/Lab-S02-Docker-dia-1.html. Aunque sea tarde, subela: tarde no baja puntos, pero sin entrega no hay calificacion.</t>
+          <t>Abrelo, escribe tu nombre completo y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>Tu p00 esta guardado en latin-1 y tu apellido con ñ sale roto.</t>
+          <t>En tu evidencia escribes docker build -t mi-sitio sin el punto final.</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Vuelve a guardarlo eligiendo codificacion UTF-8.</t>
-        </is>
-      </c>
-    </row>
+          <t>El punto es obligatorio: le dice a Docker donde buscar el Dockerfile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
@@ -3083,24 +2967,25 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 320298835</t>
+          <t>Correccion · 320152841</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320298835   ·   Por corregir: p00</t>
+          <t>Cuenta: 320152841   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: ✓      L2: ✓</t>
-        </is>
-      </c>
-    </row>
+          <t>P00: ✓      S02: ✓      L2: ✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
@@ -3116,27 +3001,28 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Tu p00 no lleva tu nombre: dice 'esta es una prueba de git'.</t>
+          <t>Tu respuesta de por que la pagina no cambio esta equivocada: dices que Docker bloquea la imagen.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Abrelo, escribe tu nombre completo y haz push.</t>
+          <t>La razon es que la imagen es inmutable: el contenedor sigue corriendo la imagen vieja, y hasta que no reconstruyes con docker build no existe una imagen nueva.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>En tu evidencia escribes docker build -t mi-sitio sin el punto final.</t>
+          <t>Tu carpeta lleva solo tu apellido.</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>El punto es obligatorio: le dice a Docker donde buscar el Dockerfile.</t>
-        </is>
-      </c>
-    </row>
+          <t>Deberia ser apellido_nombre, igual que tu rama.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
@@ -3214,24 +3100,25 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 320152841</t>
+          <t>Correccion · 320250648</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320152841   ·   Por corregir: S02</t>
+          <t>Cuenta: 320250648   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: ✓      L2: ✗</t>
-        </is>
-      </c>
-    </row>
+          <t>P00: ✓      S02: ✓      L2: ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
@@ -3247,27 +3134,28 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Tu respuesta de por que la pagina no cambio esta equivocada: dices que Docker bloquea la imagen.</t>
+          <t>Tu p00 no lleva tu nombre.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>La razon es que la imagen es inmutable: el contenedor sigue corriendo la imagen vieja, y hasta que no reconstruyes con docker build no existe una imagen nueva.</t>
+          <t>Abrelo, escribe tu nombre completo y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>Tu carpeta lleva solo tu apellido.</t>
+          <t>Tu carpeta lleva mayusculas.</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Deberia ser apellido_nombre, igual que tu rama.</t>
-        </is>
-      </c>
-    </row>
+          <t>Deberia ir en minusculas: apellido_nombre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
@@ -3335,7 +3223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -3345,24 +3233,25 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 320250648</t>
+          <t>Correccion · 319659852</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320250648   ·   Por corregir: p00</t>
+          <t>Cuenta: 319659852   ·   Por corregir: S02 · lo que quedaste de corregir</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: ✓      L2: ✓</t>
-        </is>
-      </c>
-    </row>
+          <t>P00: ✓      S02: ✓      L2: ✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
@@ -3378,78 +3267,91 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Tu p00 no lleva tu nombre.</t>
+          <t>Falta el error de puerto ocupado: no aparece en tu evidencia.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Abrelo, escribe tu nombre completo y haz push.</t>
+          <t>Levanta dos contenedores en el mismo puerto; el segundo falla con 'port is already allocated'. Pega ese texto en tu evidencia.md.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>Tu carpeta se llama Salgado_Roman con mayusculas.</t>
+          <t>Tu Dockerfile es el unico sin EXPOSE 80.</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Deberia ir en minusculas: apellido_nombre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+          <t>Agregale la linea EXPOSE 80 . Construye igual, pero documenta que el contenedor escucha en ese puerto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Tu p00 ya quedo registrada, esa ya no le muevas.</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Tu S02 ya cuenta como entregada: estas dos correcciones son para dejarla completa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>git commit -m "S02: correccion"</t>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
         <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
           <t>git push</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3476,24 +3378,25 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 319659852</t>
+          <t>Correccion · 320229264</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 319659852   ·   Por corregir: S02 · lo que quedaste de corregir</t>
+          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: ✓      L2: ✗</t>
-        </is>
-      </c>
-    </row>
+          <t>P00: ✓      S02: parcial      L2: ✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
@@ -3509,39 +3412,40 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Falta el error de puerto ocupado: no aparece en tu evidencia.</t>
+          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Levanta dos contenedores en el mismo puerto; el segundo falla con 'port is already allocated'. Pega ese texto en tu evidencia.md.</t>
+          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>Tu Dockerfile es el unico sin EXPOSE 80.</t>
+          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Agregale la linea EXPOSE 80 . Construye igual, pero documenta que el contenedor escucha en ese puerto.</t>
+          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t>Tu p00 ya quedo registrada, esa ya no le muevas.</t>
+          <t>Tu index.html no trae la tabla de 5 comandos.</t>
         </is>
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>Tu S02 ya cuenta como entregada: estas dos correcciones son para dejarla completa.</t>
-        </is>
-      </c>
-    </row>
+          <t>Esa era la mision 1: agregala.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
@@ -3609,7 +3513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -3619,24 +3523,25 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 320229264</t>
+          <t>Correccion · 320284858</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
+          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: ✗</t>
-        </is>
-      </c>
-    </row>
+          <t>P00: ✓      S02: ✓      L2: ✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
@@ -3652,90 +3557,67 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
+          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Tu index.html no trae la tabla de 5 comandos.</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Esa era la mision 1: agregala.</t>
+          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>git checkout TU-RAMA</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
+          <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3762,24 +3644,25 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 320284858</t>
+          <t>Correccion · 320224159</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
+          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: ✓      L2: ✗</t>
-        </is>
-      </c>
-    </row>
+          <t>P00: ✓      S02: parcial      L2: ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
@@ -3795,15 +3678,16 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
+          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
-        </is>
-      </c>
-    </row>
+          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="19" t="inlineStr">
         <is>
@@ -3881,24 +3765,25 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 320224159</t>
+          <t>Correccion · 320049376</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
+          <t>Cuenta: 320049376   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
-        </is>
-      </c>
-    </row>
+          <t>P00: ✓      S02: ✓      L2: ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
@@ -3914,15 +3799,16 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
+          <t>No tienes p00, que era la primera tarea de Git.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
-        </is>
-      </c>
-    </row>
+          <t>Crea entregas/tu_carpeta/p00/prueba.txt con tu nombre completo adentro y haz push. Tu S02 si esta completa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="19" t="inlineStr">
         <is>

</xml_diff>